<commit_message>
Styling Updates, Color Selection, and Step2 Mods
Adding black and white styling as well as company logo.
Added library to make picking color for formatting easier in Step 5.
Starting modifying Step 2 to incorporate if no member with exact share list.
This was a big update so there may be more I am missing.
</commit_message>
<xml_diff>
--- a/Customer_Order_Printout/Member Pick-up Details-shiny_test.xlsx
+++ b/Customer_Order_Printout/Member Pick-up Details-shiny_test.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\fair_shares_ds_projects\FS_P003_Customer_Order_List\Customer_Order_Printout\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACC09B8-FAD3-443D-A0F6-10A51D981916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7FD57CC-4806-4B72-B679-9EC99C8896AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19080" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Member Pick-up Details-shiny_te" sheetId="1" r:id="rId1"/>
-    <sheet name="Shares" sheetId="2" r:id="rId2"/>
+    <sheet name="members" sheetId="1" r:id="rId1"/>
+    <sheet name="shares" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="252">
   <si>
     <t>Pickup Site</t>
   </si>
@@ -768,6 +768,15 @@
   </si>
   <si>
     <t>Potatoes - Sweet</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Item Description</t>
   </si>
 </sst>
 </file>
@@ -1309,9 +1318,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1704,958 +1712,980 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="E4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B33" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B34" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="C35" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B36" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B37" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B38" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B39" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B40" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B41" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B42" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B43" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B44" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B45" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B46" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B47" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B48" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B49" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B50" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B51" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B52" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B53" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C53" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B54" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B55" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="C56" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="D56" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B57" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B58" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C58" t="s">
+      <c r="D58" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B59" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C59" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C59" t="s">
+      <c r="D59" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B60" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B61" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="C61" t="s">
+      <c r="D61" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="D61" t="s">
+      <c r="E61" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B62" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="C62" t="s">
+      <c r="D62" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="D62" t="s">
+      <c r="E62" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B63" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D63" t="s">
+      <c r="E63" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B64" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="C64" t="s">
+      <c r="D64" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="D64" t="s">
+      <c r="E64" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B65" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C65" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D65" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" s="1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B66" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C66" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C66" t="s">
+      <c r="D66" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B67" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C67" t="s">
+      <c r="D67" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B68" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" s="1" t="s">
         <v>77</v>
       </c>
     </row>
@@ -2682,1442 +2712,1442 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6">
-        <v>8</v>
-      </c>
-      <c r="B2" s="7" t="s">
+      <c r="A2" s="5">
+        <v>8</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C2" s="6">
-        <v>1</v>
-      </c>
-      <c r="D2" s="8" t="s">
+      <c r="C2" s="5">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G2" s="6">
-        <v>1</v>
-      </c>
-      <c r="H2" s="9"/>
-      <c r="I2" s="6">
-        <v>1</v>
-      </c>
-      <c r="J2" s="10">
+      <c r="F2" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G2" s="5">
+        <v>1</v>
+      </c>
+      <c r="H2" s="8"/>
+      <c r="I2" s="5">
+        <v>1</v>
+      </c>
+      <c r="J2" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
-        <v>8</v>
-      </c>
-      <c r="B3" s="7" t="s">
+      <c r="A3" s="5">
+        <v>8</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C3" s="6">
-        <v>1</v>
-      </c>
-      <c r="D3" s="8" t="s">
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F3" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G3" s="6">
+      <c r="F3" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G3" s="5">
         <v>2</v>
       </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="6">
-        <v>1</v>
-      </c>
-      <c r="J3" s="10">
+      <c r="H3" s="8"/>
+      <c r="I3" s="5">
+        <v>1</v>
+      </c>
+      <c r="J3" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6">
-        <v>8</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="A4" s="5">
+        <v>8</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C4" s="6">
-        <v>1</v>
-      </c>
-      <c r="D4" s="8" t="s">
+      <c r="C4" s="5">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F4" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G4" s="6">
+      <c r="F4" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G4" s="5">
         <v>3</v>
       </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="6">
-        <v>1</v>
-      </c>
-      <c r="J4" s="10">
+      <c r="H4" s="8"/>
+      <c r="I4" s="5">
+        <v>1</v>
+      </c>
+      <c r="J4" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6">
-        <v>8</v>
-      </c>
-      <c r="B5" s="7" t="s">
+      <c r="A5" s="5">
+        <v>8</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C5" s="6">
-        <v>1</v>
-      </c>
-      <c r="D5" s="8" t="s">
+      <c r="C5" s="5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G5" s="6">
+      <c r="F5" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G5" s="5">
         <v>4</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="6">
-        <v>1</v>
-      </c>
-      <c r="J5" s="10">
+      <c r="H5" s="8"/>
+      <c r="I5" s="5">
+        <v>1</v>
+      </c>
+      <c r="J5" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
-        <v>8</v>
-      </c>
-      <c r="B6" s="7" t="s">
+      <c r="A6" s="5">
+        <v>8</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C6" s="6">
-        <v>1</v>
-      </c>
-      <c r="D6" s="8" t="s">
+      <c r="C6" s="5">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G6" s="6">
+      <c r="F6" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G6" s="5">
         <v>5</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="6">
-        <v>1</v>
-      </c>
-      <c r="J6" s="10">
+      <c r="H6" s="8"/>
+      <c r="I6" s="5">
+        <v>1</v>
+      </c>
+      <c r="J6" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6">
-        <v>8</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="A7" s="5">
+        <v>8</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C7" s="6">
-        <v>1</v>
-      </c>
-      <c r="D7" s="8" t="s">
+      <c r="C7" s="5">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G7" s="6">
+      <c r="E7" s="7"/>
+      <c r="F7" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G7" s="5">
         <v>6</v>
       </c>
-      <c r="H7" s="9"/>
-      <c r="I7" s="6">
-        <v>1</v>
-      </c>
-      <c r="J7" s="10">
+      <c r="H7" s="8"/>
+      <c r="I7" s="5">
+        <v>1</v>
+      </c>
+      <c r="J7" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="6">
-        <v>8</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="5">
+        <v>8</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C8" s="6">
-        <v>1</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="C8" s="5">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G8" s="6">
+      <c r="E8" s="7"/>
+      <c r="F8" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G8" s="5">
         <v>7</v>
       </c>
-      <c r="H8" s="9"/>
-      <c r="I8" s="6">
-        <v>1</v>
-      </c>
-      <c r="J8" s="10">
+      <c r="H8" s="8"/>
+      <c r="I8" s="5">
+        <v>1</v>
+      </c>
+      <c r="J8" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="6">
-        <v>8</v>
-      </c>
-      <c r="B9" s="7" t="s">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C9" s="6">
-        <v>1</v>
-      </c>
-      <c r="D9" s="8" t="s">
+      <c r="C9" s="5">
+        <v>1</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G9" s="6">
-        <v>8</v>
-      </c>
-      <c r="H9" s="8" t="s">
+      <c r="E9" s="7"/>
+      <c r="F9" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G9" s="5">
+        <v>8</v>
+      </c>
+      <c r="H9" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="I9" s="6">
-        <v>1</v>
-      </c>
-      <c r="J9" s="10">
+      <c r="I9" s="5">
+        <v>1</v>
+      </c>
+      <c r="J9" s="9">
         <v>0.41</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
-        <v>8</v>
-      </c>
-      <c r="B10" s="7" t="s">
+      <c r="A10" s="5">
+        <v>8</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C10" s="6">
-        <v>1</v>
-      </c>
-      <c r="D10" s="8" t="s">
+      <c r="C10" s="5">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G10" s="6">
-        <v>8</v>
-      </c>
-      <c r="H10" s="8" t="s">
+      <c r="E10" s="7"/>
+      <c r="F10" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G10" s="5">
+        <v>8</v>
+      </c>
+      <c r="H10" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="I10" s="6">
-        <v>1</v>
-      </c>
-      <c r="J10" s="10">
+      <c r="I10" s="5">
+        <v>1</v>
+      </c>
+      <c r="J10" s="9">
         <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="6">
-        <v>8</v>
-      </c>
-      <c r="B11" s="7" t="s">
+      <c r="A11" s="5">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C11" s="6">
-        <v>1</v>
-      </c>
-      <c r="D11" s="8" t="s">
+      <c r="C11" s="5">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G11" s="6">
+      <c r="E11" s="7"/>
+      <c r="F11" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G11" s="5">
         <v>9</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="6">
-        <v>1</v>
-      </c>
-      <c r="J11" s="10">
+      <c r="H11" s="7"/>
+      <c r="I11" s="5">
+        <v>1</v>
+      </c>
+      <c r="J11" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="6">
-        <v>8</v>
-      </c>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="5">
+        <v>8</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C12" s="6">
-        <v>1</v>
-      </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="6">
-        <v>1</v>
-      </c>
-      <c r="J12" s="10">
+      <c r="C12" s="5">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="5">
+        <v>1</v>
+      </c>
+      <c r="J12" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="6">
-        <v>8</v>
-      </c>
-      <c r="B13" s="11" t="s">
+      <c r="A13" s="5">
+        <v>8</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="5">
         <v>2</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G13" s="6">
-        <v>1</v>
-      </c>
-      <c r="H13" s="9"/>
-      <c r="I13" s="6">
-        <v>1</v>
-      </c>
-      <c r="J13" s="10">
+      <c r="F13" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G13" s="5">
+        <v>1</v>
+      </c>
+      <c r="H13" s="8"/>
+      <c r="I13" s="5">
+        <v>1</v>
+      </c>
+      <c r="J13" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="6">
-        <v>8</v>
-      </c>
-      <c r="B14" s="11" t="s">
+      <c r="A14" s="5">
+        <v>8</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="5">
         <v>2</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F14" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G14" s="6">
+      <c r="F14" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G14" s="5">
         <v>2</v>
       </c>
-      <c r="H14" s="9"/>
-      <c r="I14" s="6">
-        <v>1</v>
-      </c>
-      <c r="J14" s="10">
+      <c r="H14" s="8"/>
+      <c r="I14" s="5">
+        <v>1</v>
+      </c>
+      <c r="J14" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="6">
-        <v>8</v>
-      </c>
-      <c r="B15" s="11" t="s">
+      <c r="A15" s="5">
+        <v>8</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="5">
         <v>2</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F15" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G15" s="6">
+      <c r="F15" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G15" s="5">
         <v>3</v>
       </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="6">
-        <v>1</v>
-      </c>
-      <c r="J15" s="10">
+      <c r="H15" s="7"/>
+      <c r="I15" s="5">
+        <v>1</v>
+      </c>
+      <c r="J15" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="6">
-        <v>8</v>
-      </c>
-      <c r="B16" s="11" t="s">
+      <c r="A16" s="5">
+        <v>8</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="5">
         <v>2</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G16" s="6">
+      <c r="E16" s="7"/>
+      <c r="F16" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G16" s="5">
         <v>4</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="I16" s="6">
-        <v>1</v>
-      </c>
-      <c r="J16" s="10">
+      <c r="I16" s="5">
+        <v>1</v>
+      </c>
+      <c r="J16" s="9">
         <v>0.44500000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="6">
-        <v>8</v>
-      </c>
-      <c r="B17" s="11" t="s">
+      <c r="A17" s="5">
+        <v>8</v>
+      </c>
+      <c r="B17" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="5">
         <v>2</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G17" s="6">
+      <c r="E17" s="7"/>
+      <c r="F17" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G17" s="5">
         <v>4</v>
       </c>
-      <c r="H17" s="8" t="s">
+      <c r="H17" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="5">
         <v>2</v>
       </c>
-      <c r="J17" s="10">
+      <c r="J17" s="9">
         <v>0.54</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="6">
-        <v>8</v>
-      </c>
-      <c r="B18" s="11" t="s">
+      <c r="A18" s="5">
+        <v>8</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C18" s="6">
+      <c r="C18" s="5">
         <v>2</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G18" s="6">
+      <c r="E18" s="7"/>
+      <c r="F18" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G18" s="5">
         <v>5</v>
       </c>
-      <c r="H18" s="9"/>
-      <c r="I18" s="6">
-        <v>1</v>
-      </c>
-      <c r="J18" s="10">
+      <c r="H18" s="8"/>
+      <c r="I18" s="5">
+        <v>1</v>
+      </c>
+      <c r="J18" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="6">
-        <v>8</v>
-      </c>
-      <c r="B19" s="11" t="s">
+      <c r="A19" s="5">
+        <v>8</v>
+      </c>
+      <c r="B19" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="5">
         <v>2</v>
       </c>
-      <c r="D19" s="9"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="6">
-        <v>1</v>
-      </c>
-      <c r="J19" s="10">
+      <c r="D19" s="8"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="5">
+        <v>1</v>
+      </c>
+      <c r="J19" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="6">
-        <v>8</v>
-      </c>
-      <c r="B20" s="12" t="s">
+      <c r="A20" s="5">
+        <v>8</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="5">
         <v>3</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="E20" s="8" t="s">
+      <c r="E20" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F20" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G20" s="6">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9"/>
-      <c r="I20" s="6">
-        <v>1</v>
-      </c>
-      <c r="J20" s="10">
+      <c r="F20" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G20" s="5">
+        <v>1</v>
+      </c>
+      <c r="H20" s="8"/>
+      <c r="I20" s="5">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="6">
-        <v>8</v>
-      </c>
-      <c r="B21" s="12" t="s">
+      <c r="A21" s="5">
+        <v>8</v>
+      </c>
+      <c r="B21" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="5">
         <v>3</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F21" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G21" s="6">
+      <c r="F21" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G21" s="5">
         <v>2</v>
       </c>
-      <c r="H21" s="9"/>
-      <c r="I21" s="6">
-        <v>1</v>
-      </c>
-      <c r="J21" s="10">
+      <c r="H21" s="8"/>
+      <c r="I21" s="5">
+        <v>1</v>
+      </c>
+      <c r="J21" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="6">
-        <v>8</v>
-      </c>
-      <c r="B22" s="12" t="s">
+      <c r="A22" s="5">
+        <v>8</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="5">
         <v>3</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F22" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G22" s="6">
+      <c r="F22" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G22" s="5">
         <v>3</v>
       </c>
-      <c r="H22" s="9"/>
-      <c r="I22" s="6">
-        <v>1</v>
-      </c>
-      <c r="J22" s="10">
+      <c r="H22" s="8"/>
+      <c r="I22" s="5">
+        <v>1</v>
+      </c>
+      <c r="J22" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="6">
-        <v>8</v>
-      </c>
-      <c r="B23" s="12" t="s">
+      <c r="A23" s="5">
+        <v>8</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="5">
         <v>3</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F23" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G23" s="6">
+      <c r="F23" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G23" s="5">
         <v>4</v>
       </c>
-      <c r="H23" s="9"/>
-      <c r="I23" s="6">
-        <v>1</v>
-      </c>
-      <c r="J23" s="10">
+      <c r="H23" s="8"/>
+      <c r="I23" s="5">
+        <v>1</v>
+      </c>
+      <c r="J23" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="6">
-        <v>8</v>
-      </c>
-      <c r="B24" s="12" t="s">
+      <c r="A24" s="5">
+        <v>8</v>
+      </c>
+      <c r="B24" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="5">
         <v>3</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G24" s="6">
+      <c r="E24" s="7"/>
+      <c r="F24" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G24" s="5">
         <v>5</v>
       </c>
-      <c r="H24" s="9"/>
-      <c r="I24" s="6">
-        <v>1</v>
-      </c>
-      <c r="J24" s="10">
+      <c r="H24" s="8"/>
+      <c r="I24" s="5">
+        <v>1</v>
+      </c>
+      <c r="J24" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="6">
-        <v>8</v>
-      </c>
-      <c r="B25" s="12" t="s">
+      <c r="A25" s="5">
+        <v>8</v>
+      </c>
+      <c r="B25" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="5">
         <v>3</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G25" s="6">
+      <c r="E25" s="7"/>
+      <c r="F25" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G25" s="5">
         <v>6</v>
       </c>
-      <c r="H25" s="8" t="s">
+      <c r="H25" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="I25" s="6">
-        <v>1</v>
-      </c>
-      <c r="J25" s="10">
+      <c r="I25" s="5">
+        <v>1</v>
+      </c>
+      <c r="J25" s="9">
         <v>0.62</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="6">
-        <v>8</v>
-      </c>
-      <c r="B26" s="12" t="s">
+      <c r="A26" s="5">
+        <v>8</v>
+      </c>
+      <c r="B26" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="5">
         <v>3</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G26" s="6">
+      <c r="E26" s="7"/>
+      <c r="F26" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G26" s="5">
         <v>6</v>
       </c>
-      <c r="H26" s="8" t="s">
+      <c r="H26" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="I26" s="6">
-        <v>1</v>
-      </c>
-      <c r="J26" s="10">
+      <c r="I26" s="5">
+        <v>1</v>
+      </c>
+      <c r="J26" s="9">
         <v>0.38</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="6">
-        <v>8</v>
-      </c>
-      <c r="B27" s="12" t="s">
+      <c r="A27" s="5">
+        <v>8</v>
+      </c>
+      <c r="B27" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="5">
         <v>3</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="7" t="s">
         <v>233</v>
       </c>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G27" s="6">
+      <c r="E27" s="7"/>
+      <c r="F27" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G27" s="5">
         <v>7</v>
       </c>
-      <c r="H27" s="9"/>
-      <c r="I27" s="6">
-        <v>1</v>
-      </c>
-      <c r="J27" s="10">
+      <c r="H27" s="8"/>
+      <c r="I27" s="5">
+        <v>1</v>
+      </c>
+      <c r="J27" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="6">
-        <v>8</v>
-      </c>
-      <c r="B28" s="12" t="s">
+      <c r="A28" s="5">
+        <v>8</v>
+      </c>
+      <c r="B28" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="C28" s="6">
+      <c r="C28" s="5">
         <v>3</v>
       </c>
-      <c r="D28" s="9"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="6">
-        <v>1</v>
-      </c>
-      <c r="J28" s="10">
+      <c r="D28" s="8"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="5">
+        <v>1</v>
+      </c>
+      <c r="J28" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="6">
-        <v>8</v>
-      </c>
-      <c r="B29" s="3" t="s">
+      <c r="A29" s="5">
+        <v>8</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="5">
         <v>4</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="E29" s="8" t="s">
+      <c r="E29" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F29" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G29" s="6">
-        <v>1</v>
-      </c>
-      <c r="H29" s="8"/>
-      <c r="I29" s="6">
-        <v>1</v>
-      </c>
-      <c r="J29" s="10">
+      <c r="F29" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G29" s="5">
+        <v>1</v>
+      </c>
+      <c r="H29" s="7"/>
+      <c r="I29" s="5">
+        <v>1</v>
+      </c>
+      <c r="J29" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="6">
-        <v>8</v>
-      </c>
-      <c r="B30" s="3" t="s">
+      <c r="A30" s="5">
+        <v>8</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="5">
         <v>4</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="D30" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F30" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G30" s="6">
+      <c r="F30" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G30" s="5">
         <v>2</v>
       </c>
-      <c r="H30" s="8"/>
-      <c r="I30" s="6">
-        <v>1</v>
-      </c>
-      <c r="J30" s="10">
+      <c r="H30" s="7"/>
+      <c r="I30" s="5">
+        <v>1</v>
+      </c>
+      <c r="J30" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="6">
-        <v>8</v>
-      </c>
-      <c r="B31" s="3" t="s">
+      <c r="A31" s="5">
+        <v>8</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="5">
         <v>4</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="D31" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="E31" s="8" t="s">
+      <c r="E31" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F31" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G31" s="6">
+      <c r="F31" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G31" s="5">
         <v>3</v>
       </c>
-      <c r="H31" s="8"/>
-      <c r="I31" s="6">
-        <v>1</v>
-      </c>
-      <c r="J31" s="10">
+      <c r="H31" s="7"/>
+      <c r="I31" s="5">
+        <v>1</v>
+      </c>
+      <c r="J31" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="6">
-        <v>8</v>
-      </c>
-      <c r="B32" s="3" t="s">
+      <c r="A32" s="5">
+        <v>8</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C32" s="6">
+      <c r="C32" s="5">
         <v>4</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="D32" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="E32" s="8" t="s">
+      <c r="E32" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F32" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G32" s="6">
+      <c r="F32" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G32" s="5">
         <v>4</v>
       </c>
-      <c r="H32" s="9"/>
-      <c r="I32" s="6">
-        <v>1</v>
-      </c>
-      <c r="J32" s="10">
+      <c r="H32" s="8"/>
+      <c r="I32" s="5">
+        <v>1</v>
+      </c>
+      <c r="J32" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="6">
-        <v>8</v>
-      </c>
-      <c r="B33" s="3" t="s">
+      <c r="A33" s="5">
+        <v>8</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C33" s="6">
+      <c r="C33" s="5">
         <v>4</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="E33" s="8" t="s">
+      <c r="E33" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F33" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G33" s="6">
+      <c r="F33" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G33" s="5">
         <v>5</v>
       </c>
-      <c r="H33" s="9"/>
-      <c r="I33" s="6">
-        <v>1</v>
-      </c>
-      <c r="J33" s="10">
+      <c r="H33" s="8"/>
+      <c r="I33" s="5">
+        <v>1</v>
+      </c>
+      <c r="J33" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="6">
-        <v>8</v>
-      </c>
-      <c r="B34" s="3" t="s">
+      <c r="A34" s="5">
+        <v>8</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C34" s="6">
+      <c r="C34" s="5">
         <v>4</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="D34" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E34" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F34" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G34" s="6">
+      <c r="F34" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G34" s="5">
         <v>6</v>
       </c>
-      <c r="H34" s="9"/>
-      <c r="I34" s="6">
-        <v>1</v>
-      </c>
-      <c r="J34" s="10">
+      <c r="H34" s="8"/>
+      <c r="I34" s="5">
+        <v>1</v>
+      </c>
+      <c r="J34" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="6">
-        <v>8</v>
-      </c>
-      <c r="B35" s="3" t="s">
+      <c r="A35" s="5">
+        <v>8</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C35" s="6">
+      <c r="C35" s="5">
         <v>4</v>
       </c>
-      <c r="D35" s="8" t="s">
+      <c r="D35" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G35" s="6">
+      <c r="E35" s="7"/>
+      <c r="F35" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G35" s="5">
         <v>7</v>
       </c>
-      <c r="H35" s="9"/>
-      <c r="I35" s="6">
-        <v>1</v>
-      </c>
-      <c r="J35" s="10">
+      <c r="H35" s="8"/>
+      <c r="I35" s="5">
+        <v>1</v>
+      </c>
+      <c r="J35" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="6">
-        <v>8</v>
-      </c>
-      <c r="B36" s="3" t="s">
+      <c r="A36" s="5">
+        <v>8</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C36" s="6">
+      <c r="C36" s="5">
         <v>4</v>
       </c>
-      <c r="D36" s="8" t="s">
+      <c r="D36" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G36" s="6">
-        <v>8</v>
-      </c>
-      <c r="H36" s="8" t="s">
+      <c r="E36" s="7"/>
+      <c r="F36" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G36" s="5">
+        <v>8</v>
+      </c>
+      <c r="H36" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="I36" s="6">
-        <v>1</v>
-      </c>
-      <c r="J36" s="10">
+      <c r="I36" s="5">
+        <v>1</v>
+      </c>
+      <c r="J36" s="9">
         <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="6">
-        <v>8</v>
-      </c>
-      <c r="B37" s="3" t="s">
+      <c r="A37" s="5">
+        <v>8</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C37" s="6">
+      <c r="C37" s="5">
         <v>4</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D37" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G37" s="6">
-        <v>8</v>
-      </c>
-      <c r="H37" s="8" t="s">
+      <c r="E37" s="7"/>
+      <c r="F37" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G37" s="5">
+        <v>8</v>
+      </c>
+      <c r="H37" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="I37" s="6">
-        <v>1</v>
-      </c>
-      <c r="J37" s="10">
+      <c r="I37" s="5">
+        <v>1</v>
+      </c>
+      <c r="J37" s="9">
         <v>0.41</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="6">
-        <v>8</v>
-      </c>
-      <c r="B38" s="3" t="s">
+      <c r="A38" s="5">
+        <v>8</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C38" s="6">
+      <c r="C38" s="5">
         <v>4</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="D38" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G38" s="6">
+      <c r="E38" s="7"/>
+      <c r="F38" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G38" s="5">
         <v>9</v>
       </c>
-      <c r="H38" s="9"/>
-      <c r="I38" s="6">
-        <v>1</v>
-      </c>
-      <c r="J38" s="10">
+      <c r="H38" s="8"/>
+      <c r="I38" s="5">
+        <v>1</v>
+      </c>
+      <c r="J38" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="6">
-        <v>8</v>
-      </c>
-      <c r="B39" s="3" t="s">
+      <c r="A39" s="5">
+        <v>8</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C39" s="6">
+      <c r="C39" s="5">
         <v>4</v>
       </c>
-      <c r="D39" s="9"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="6">
-        <v>1</v>
-      </c>
-      <c r="J39" s="10">
+      <c r="D39" s="8"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="5">
+        <v>1</v>
+      </c>
+      <c r="J39" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="6">
-        <v>8</v>
-      </c>
-      <c r="B40" s="13" t="s">
+      <c r="A40" s="5">
+        <v>8</v>
+      </c>
+      <c r="B40" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C40" s="6">
+      <c r="C40" s="5">
         <v>5</v>
       </c>
-      <c r="D40" s="8" t="s">
+      <c r="D40" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="E40" s="8" t="s">
+      <c r="E40" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F40" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G40" s="6">
-        <v>1</v>
-      </c>
-      <c r="H40" s="9"/>
-      <c r="I40" s="6">
-        <v>1</v>
-      </c>
-      <c r="J40" s="10">
+      <c r="F40" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G40" s="5">
+        <v>1</v>
+      </c>
+      <c r="H40" s="8"/>
+      <c r="I40" s="5">
+        <v>1</v>
+      </c>
+      <c r="J40" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="6">
-        <v>8</v>
-      </c>
-      <c r="B41" s="13" t="s">
+      <c r="A41" s="5">
+        <v>8</v>
+      </c>
+      <c r="B41" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C41" s="6">
+      <c r="C41" s="5">
         <v>5</v>
       </c>
-      <c r="D41" s="8" t="s">
+      <c r="D41" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="E41" s="8" t="s">
+      <c r="E41" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F41" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G41" s="6">
+      <c r="F41" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G41" s="5">
         <v>2</v>
       </c>
-      <c r="H41" s="9"/>
-      <c r="I41" s="6">
-        <v>1</v>
-      </c>
-      <c r="J41" s="10">
+      <c r="H41" s="8"/>
+      <c r="I41" s="5">
+        <v>1</v>
+      </c>
+      <c r="J41" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="6">
-        <v>8</v>
-      </c>
-      <c r="B42" s="13" t="s">
+      <c r="A42" s="5">
+        <v>8</v>
+      </c>
+      <c r="B42" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C42" s="6">
+      <c r="C42" s="5">
         <v>5</v>
       </c>
-      <c r="D42" s="8" t="s">
+      <c r="D42" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="E42" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F42" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G42" s="6">
+      <c r="F42" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G42" s="5">
         <v>3</v>
       </c>
-      <c r="H42" s="9"/>
-      <c r="I42" s="6">
-        <v>1</v>
-      </c>
-      <c r="J42" s="10">
+      <c r="H42" s="8"/>
+      <c r="I42" s="5">
+        <v>1</v>
+      </c>
+      <c r="J42" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="6">
-        <v>8</v>
-      </c>
-      <c r="B43" s="13" t="s">
+      <c r="A43" s="5">
+        <v>8</v>
+      </c>
+      <c r="B43" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C43" s="6">
+      <c r="C43" s="5">
         <v>5</v>
       </c>
-      <c r="D43" s="14" t="s">
+      <c r="D43" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="E43" s="8" t="s">
+      <c r="E43" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F43" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G43" s="6">
+      <c r="F43" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G43" s="5">
         <v>4</v>
       </c>
-      <c r="H43" s="9"/>
-      <c r="I43" s="6">
-        <v>1</v>
-      </c>
-      <c r="J43" s="10">
+      <c r="H43" s="8"/>
+      <c r="I43" s="5">
+        <v>1</v>
+      </c>
+      <c r="J43" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="6">
-        <v>8</v>
-      </c>
-      <c r="B44" s="13" t="s">
+      <c r="A44" s="5">
+        <v>8</v>
+      </c>
+      <c r="B44" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C44" s="6">
+      <c r="C44" s="5">
         <v>5</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="D44" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="E44" s="8" t="s">
+      <c r="E44" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="F44" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G44" s="6">
+      <c r="F44" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G44" s="5">
         <v>5</v>
       </c>
-      <c r="H44" s="9"/>
-      <c r="I44" s="6">
-        <v>1</v>
-      </c>
-      <c r="J44" s="10">
+      <c r="H44" s="8"/>
+      <c r="I44" s="5">
+        <v>1</v>
+      </c>
+      <c r="J44" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="6">
-        <v>8</v>
-      </c>
-      <c r="B45" s="13" t="s">
+      <c r="A45" s="5">
+        <v>8</v>
+      </c>
+      <c r="B45" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C45" s="6">
+      <c r="C45" s="5">
         <v>5</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="D45" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G45" s="6">
+      <c r="E45" s="7"/>
+      <c r="F45" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G45" s="5">
         <v>6</v>
       </c>
-      <c r="H45" s="9"/>
-      <c r="I45" s="6">
-        <v>1</v>
-      </c>
-      <c r="J45" s="10">
+      <c r="H45" s="8"/>
+      <c r="I45" s="5">
+        <v>1</v>
+      </c>
+      <c r="J45" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="6">
-        <v>8</v>
-      </c>
-      <c r="B46" s="13" t="s">
+      <c r="A46" s="5">
+        <v>8</v>
+      </c>
+      <c r="B46" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C46" s="6">
+      <c r="C46" s="5">
         <v>5</v>
       </c>
-      <c r="D46" s="8" t="s">
+      <c r="D46" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="E46" s="8"/>
-      <c r="F46" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G46" s="6">
+      <c r="E46" s="7"/>
+      <c r="F46" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G46" s="5">
         <v>7</v>
       </c>
-      <c r="H46" s="8" t="s">
+      <c r="H46" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="I46" s="6">
-        <v>1</v>
-      </c>
-      <c r="J46" s="10">
+      <c r="I46" s="5">
+        <v>1</v>
+      </c>
+      <c r="J46" s="9">
         <v>0.4</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="6">
-        <v>8</v>
-      </c>
-      <c r="B47" s="13" t="s">
+      <c r="A47" s="5">
+        <v>8</v>
+      </c>
+      <c r="B47" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C47" s="6">
+      <c r="C47" s="5">
         <v>5</v>
       </c>
-      <c r="D47" s="8" t="s">
+      <c r="D47" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G47" s="6">
+      <c r="E47" s="7"/>
+      <c r="F47" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G47" s="5">
         <v>7</v>
       </c>
-      <c r="H47" s="8" t="s">
+      <c r="H47" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="I47" s="6">
-        <v>1</v>
-      </c>
-      <c r="J47" s="10">
+      <c r="I47" s="5">
+        <v>1</v>
+      </c>
+      <c r="J47" s="9">
         <v>0.6</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="6">
-        <v>8</v>
-      </c>
-      <c r="B48" s="13" t="s">
+      <c r="A48" s="5">
+        <v>8</v>
+      </c>
+      <c r="B48" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C48" s="6">
+      <c r="C48" s="5">
         <v>5</v>
       </c>
-      <c r="D48" s="8" t="s">
+      <c r="D48" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="E48" s="8"/>
-      <c r="F48" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G48" s="6">
-        <v>8</v>
-      </c>
-      <c r="H48" s="8"/>
-      <c r="I48" s="6">
-        <v>1</v>
-      </c>
-      <c r="J48" s="10">
+      <c r="E48" s="7"/>
+      <c r="F48" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G48" s="5">
+        <v>8</v>
+      </c>
+      <c r="H48" s="7"/>
+      <c r="I48" s="5">
+        <v>1</v>
+      </c>
+      <c r="J48" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="6">
-        <v>8</v>
-      </c>
-      <c r="B49" s="13" t="s">
+      <c r="A49" s="5">
+        <v>8</v>
+      </c>
+      <c r="B49" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C49" s="6">
+      <c r="C49" s="5">
         <v>5</v>
       </c>
-      <c r="D49" s="8" t="s">
+      <c r="D49" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="G49" s="6">
+      <c r="E49" s="7"/>
+      <c r="F49" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G49" s="5">
         <v>9</v>
       </c>
-      <c r="H49" s="8"/>
-      <c r="I49" s="6">
-        <v>1</v>
-      </c>
-      <c r="J49" s="10">
+      <c r="H49" s="7"/>
+      <c r="I49" s="5">
+        <v>1</v>
+      </c>
+      <c r="J49" s="9">
         <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="6">
-        <v>8</v>
-      </c>
-      <c r="B50" s="13" t="s">
+      <c r="A50" s="5">
+        <v>8</v>
+      </c>
+      <c r="B50" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="C50" s="6">
+      <c r="C50" s="5">
         <v>5</v>
       </c>
-      <c r="D50" s="8"/>
-      <c r="E50" s="8"/>
-      <c r="F50" s="8"/>
-      <c r="G50" s="6"/>
-      <c r="H50" s="9"/>
-      <c r="I50" s="6">
-        <v>1</v>
-      </c>
-      <c r="J50" s="10">
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="5">
+        <v>1</v>
+      </c>
+      <c r="J50" s="9">
         <v>1</v>
       </c>
     </row>

</xml_diff>